<commit_message>
Cambios en la estructura, actualizacion del mapeo e integracion de eliminar columnas de manera dinamica
</commit_message>
<xml_diff>
--- a/public/Formato facturacion - final.xlsx
+++ b/public/Formato facturacion - final.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cristian\Documents\S&amp;P\Documentos automatizacion\EOR\Web facturación\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cristian\Documents\S&amp;P\Documentos automatizacion\EOR\Web facturación\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{73F649BE-A081-4D4D-B4E1-841270FE524D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C7958E1-6F9D-4C34-9320-9A2B95D7AAE5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{7C2F0237-C030-49A0-B1F1-0009A5922E79}"/>
   </bookViews>
@@ -558,21 +558,6 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="2" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="3" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="4" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="2" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -645,6 +630,21 @@
     </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="2" applyFont="1"/>
     <xf numFmtId="166" fontId="6" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="2" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="3" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="4" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Millares" xfId="1" builtinId="3"/>
@@ -1133,565 +1133,565 @@
       <c r="AE2" s="5"/>
       <c r="AF2" s="9"/>
       <c r="AG2" s="10"/>
-      <c r="AH2" s="11" t="s">
+      <c r="AH2" s="37" t="s">
         <v>1</v>
       </c>
-      <c r="AI2" s="12"/>
-      <c r="AJ2" s="12"/>
-      <c r="AK2" s="12"/>
-      <c r="AL2" s="12"/>
-      <c r="AM2" s="12"/>
-      <c r="AN2" s="13"/>
-      <c r="AP2" s="11" t="s">
+      <c r="AI2" s="38"/>
+      <c r="AJ2" s="38"/>
+      <c r="AK2" s="38"/>
+      <c r="AL2" s="38"/>
+      <c r="AM2" s="38"/>
+      <c r="AN2" s="39"/>
+      <c r="AP2" s="37" t="s">
         <v>2</v>
       </c>
-      <c r="AQ2" s="14"/>
-      <c r="AR2" s="15"/>
-      <c r="AS2" s="16"/>
+      <c r="AQ2" s="40"/>
+      <c r="AR2" s="41"/>
+      <c r="AS2" s="11"/>
       <c r="AT2" s="10"/>
-      <c r="AU2" s="11" t="s">
+      <c r="AU2" s="37" t="s">
         <v>3</v>
       </c>
-      <c r="AV2" s="14"/>
-      <c r="AW2" s="14"/>
-      <c r="AX2" s="14"/>
-      <c r="AY2" s="14"/>
-      <c r="AZ2" s="15"/>
+      <c r="AV2" s="40"/>
+      <c r="AW2" s="40"/>
+      <c r="AX2" s="40"/>
+      <c r="AY2" s="40"/>
+      <c r="AZ2" s="41"/>
       <c r="BA2" s="10"/>
-      <c r="BB2" s="11" t="s">
+      <c r="BB2" s="37" t="s">
         <v>4</v>
       </c>
-      <c r="BC2" s="12"/>
-      <c r="BD2" s="12"/>
-      <c r="BE2" s="12"/>
-      <c r="BF2" s="12"/>
-      <c r="BG2" s="12"/>
-      <c r="BH2" s="12"/>
-      <c r="BI2" s="12"/>
-      <c r="BJ2" s="12"/>
-      <c r="BK2" s="12"/>
-      <c r="BL2" s="17" t="e">
+      <c r="BC2" s="38"/>
+      <c r="BD2" s="38"/>
+      <c r="BE2" s="38"/>
+      <c r="BF2" s="38"/>
+      <c r="BG2" s="38"/>
+      <c r="BH2" s="38"/>
+      <c r="BI2" s="38"/>
+      <c r="BJ2" s="38"/>
+      <c r="BK2" s="38"/>
+      <c r="BL2" s="12" t="e">
         <f>1/BG4</f>
         <v>#DIV/0!</v>
       </c>
     </row>
     <row r="3" spans="1:65" ht="48.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="18" t="s">
+      <c r="A3" s="13" t="s">
         <v>5</v>
       </c>
-      <c r="B3" s="18" t="s">
+      <c r="B3" s="13" t="s">
         <v>6</v>
       </c>
-      <c r="C3" s="18" t="s">
+      <c r="C3" s="13" t="s">
         <v>7</v>
       </c>
-      <c r="D3" s="18" t="s">
+      <c r="D3" s="13" t="s">
         <v>8</v>
       </c>
-      <c r="E3" s="18" t="s">
+      <c r="E3" s="13" t="s">
         <v>9</v>
       </c>
-      <c r="F3" s="18" t="s">
+      <c r="F3" s="13" t="s">
         <v>10</v>
       </c>
-      <c r="G3" s="18" t="s">
+      <c r="G3" s="13" t="s">
         <v>11</v>
       </c>
-      <c r="H3" s="19" t="s">
+      <c r="H3" s="14" t="s">
         <v>12</v>
       </c>
-      <c r="I3" s="19" t="s">
+      <c r="I3" s="14" t="s">
         <v>13</v>
       </c>
-      <c r="J3" s="19" t="s">
+      <c r="J3" s="14" t="s">
         <v>14</v>
       </c>
-      <c r="K3" s="18" t="s">
+      <c r="K3" s="13" t="s">
         <v>15</v>
       </c>
-      <c r="L3" s="18" t="s">
+      <c r="L3" s="13" t="s">
         <v>16</v>
       </c>
-      <c r="M3" s="18" t="s">
+      <c r="M3" s="13" t="s">
         <v>17</v>
       </c>
-      <c r="N3" s="18" t="s">
+      <c r="N3" s="13" t="s">
         <v>18</v>
       </c>
-      <c r="O3" s="18" t="s">
+      <c r="O3" s="13" t="s">
         <v>19</v>
       </c>
-      <c r="P3" s="18" t="s">
+      <c r="P3" s="13" t="s">
         <v>20</v>
       </c>
-      <c r="Q3" s="18" t="s">
+      <c r="Q3" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="R3" s="20" t="s">
+      <c r="R3" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="S3" s="20" t="s">
+      <c r="S3" s="15" t="s">
         <v>23</v>
       </c>
-      <c r="T3" s="21" t="s">
+      <c r="T3" s="16" t="s">
         <v>24</v>
       </c>
-      <c r="U3" s="21" t="s">
+      <c r="U3" s="16" t="s">
         <v>25</v>
       </c>
-      <c r="V3" s="18" t="s">
+      <c r="V3" s="13" t="s">
         <v>26</v>
       </c>
-      <c r="W3" s="21" t="s">
+      <c r="W3" s="16" t="s">
         <v>27</v>
       </c>
-      <c r="X3" s="21" t="s">
+      <c r="X3" s="16" t="s">
         <v>28</v>
       </c>
-      <c r="Y3" s="21" t="s">
+      <c r="Y3" s="16" t="s">
         <v>29</v>
       </c>
-      <c r="Z3" s="21" t="s">
+      <c r="Z3" s="16" t="s">
         <v>30</v>
       </c>
-      <c r="AA3" s="21" t="s">
+      <c r="AA3" s="16" t="s">
         <v>31</v>
       </c>
-      <c r="AB3" s="21" t="s">
+      <c r="AB3" s="16" t="s">
         <v>32</v>
       </c>
-      <c r="AC3" s="21" t="s">
+      <c r="AC3" s="16" t="s">
         <v>33</v>
       </c>
-      <c r="AD3" s="21" t="s">
+      <c r="AD3" s="16" t="s">
         <v>34</v>
       </c>
-      <c r="AE3" s="21" t="s">
+      <c r="AE3" s="16" t="s">
         <v>35</v>
       </c>
-      <c r="AF3" s="18" t="s">
+      <c r="AF3" s="13" t="s">
         <v>36</v>
       </c>
-      <c r="AG3" s="22"/>
-      <c r="AH3" s="21" t="s">
+      <c r="AG3" s="17"/>
+      <c r="AH3" s="16" t="s">
         <v>37</v>
       </c>
-      <c r="AI3" s="21" t="s">
+      <c r="AI3" s="16" t="s">
         <v>38</v>
       </c>
-      <c r="AJ3" s="21" t="s">
+      <c r="AJ3" s="16" t="s">
         <v>39</v>
       </c>
-      <c r="AK3" s="21" t="s">
+      <c r="AK3" s="16" t="s">
         <v>40</v>
       </c>
-      <c r="AL3" s="21" t="s">
+      <c r="AL3" s="16" t="s">
         <v>41</v>
       </c>
-      <c r="AM3" s="21" t="s">
+      <c r="AM3" s="16" t="s">
         <v>42</v>
       </c>
-      <c r="AN3" s="21" t="s">
+      <c r="AN3" s="16" t="s">
         <v>43</v>
       </c>
-      <c r="AP3" s="21" t="s">
+      <c r="AP3" s="16" t="s">
         <v>44</v>
       </c>
-      <c r="AQ3" s="21" t="s">
+      <c r="AQ3" s="16" t="s">
         <v>45</v>
       </c>
-      <c r="AR3" s="21" t="s">
+      <c r="AR3" s="16" t="s">
         <v>46</v>
       </c>
-      <c r="AS3" s="21" t="s">
+      <c r="AS3" s="16" t="s">
         <v>43</v>
       </c>
-      <c r="AT3" s="21" t="s">
+      <c r="AT3" s="16" t="s">
         <v>47</v>
       </c>
-      <c r="AU3" s="21" t="s">
+      <c r="AU3" s="16" t="s">
         <v>48</v>
       </c>
-      <c r="AV3" s="21" t="s">
+      <c r="AV3" s="16" t="s">
         <v>49</v>
       </c>
-      <c r="AW3" s="21" t="s">
+      <c r="AW3" s="16" t="s">
         <v>50</v>
       </c>
-      <c r="AX3" s="21" t="s">
+      <c r="AX3" s="16" t="s">
         <v>51</v>
       </c>
-      <c r="AY3" s="21" t="s">
+      <c r="AY3" s="16" t="s">
         <v>52</v>
       </c>
-      <c r="AZ3" s="21" t="s">
+      <c r="AZ3" s="16" t="s">
         <v>43</v>
       </c>
-      <c r="BA3" s="22"/>
-      <c r="BB3" s="21" t="s">
+      <c r="BA3" s="17"/>
+      <c r="BB3" s="16" t="s">
         <v>53</v>
       </c>
-      <c r="BC3" s="21" t="s">
+      <c r="BC3" s="16" t="s">
         <v>54</v>
       </c>
-      <c r="BD3" s="21" t="s">
+      <c r="BD3" s="16" t="s">
         <v>55</v>
       </c>
-      <c r="BE3" s="21" t="s">
+      <c r="BE3" s="16" t="s">
         <v>56</v>
       </c>
-      <c r="BF3" s="21" t="s">
+      <c r="BF3" s="16" t="s">
         <v>57</v>
       </c>
-      <c r="BG3" s="21" t="s">
+      <c r="BG3" s="16" t="s">
         <v>58</v>
       </c>
-      <c r="BH3" s="21" t="s">
+      <c r="BH3" s="16" t="s">
         <v>59</v>
       </c>
-      <c r="BI3" s="21" t="s">
+      <c r="BI3" s="16" t="s">
         <v>60</v>
       </c>
-      <c r="BJ3" s="21" t="s">
+      <c r="BJ3" s="16" t="s">
         <v>61</v>
       </c>
-      <c r="BK3" s="21" t="s">
+      <c r="BK3" s="16" t="s">
         <v>62</v>
       </c>
-      <c r="BL3" s="21" t="s">
+      <c r="BL3" s="16" t="s">
         <v>63</v>
       </c>
-      <c r="BM3" s="21" t="s">
+      <c r="BM3" s="16" t="s">
         <v>64</v>
       </c>
     </row>
     <row r="4" spans="1:65" x14ac:dyDescent="0.3">
-      <c r="A4" s="23"/>
-      <c r="B4" s="23"/>
-      <c r="C4" s="23"/>
-      <c r="D4" s="24"/>
-      <c r="E4" s="24"/>
-      <c r="F4" s="23"/>
-      <c r="G4" s="23"/>
-      <c r="H4" s="25"/>
-      <c r="I4" s="25"/>
-      <c r="J4" s="26"/>
-      <c r="K4" s="25"/>
-      <c r="L4" s="25"/>
-      <c r="M4" s="27"/>
-      <c r="N4" s="27"/>
-      <c r="O4" s="27"/>
-      <c r="P4" s="27"/>
-      <c r="Q4" s="27"/>
-      <c r="R4" s="27"/>
-      <c r="S4" s="27"/>
-      <c r="T4" s="27"/>
-      <c r="U4" s="27"/>
-      <c r="V4" s="27"/>
-      <c r="W4" s="27"/>
-      <c r="X4" s="27"/>
-      <c r="Y4" s="27"/>
-      <c r="Z4" s="27"/>
-      <c r="AA4" s="27"/>
-      <c r="AB4" s="27"/>
-      <c r="AC4" s="27"/>
-      <c r="AD4" s="27"/>
-      <c r="AE4" s="27"/>
-      <c r="AF4" s="28">
+      <c r="A4" s="18"/>
+      <c r="B4" s="18"/>
+      <c r="C4" s="18"/>
+      <c r="D4" s="19"/>
+      <c r="E4" s="19"/>
+      <c r="F4" s="18"/>
+      <c r="G4" s="18"/>
+      <c r="H4" s="20"/>
+      <c r="I4" s="20"/>
+      <c r="J4" s="21"/>
+      <c r="K4" s="20"/>
+      <c r="L4" s="20"/>
+      <c r="M4" s="22"/>
+      <c r="N4" s="22"/>
+      <c r="O4" s="22"/>
+      <c r="P4" s="22"/>
+      <c r="Q4" s="22"/>
+      <c r="R4" s="22"/>
+      <c r="S4" s="22"/>
+      <c r="T4" s="22"/>
+      <c r="U4" s="22"/>
+      <c r="V4" s="22"/>
+      <c r="W4" s="22"/>
+      <c r="X4" s="22"/>
+      <c r="Y4" s="22"/>
+      <c r="Z4" s="22"/>
+      <c r="AA4" s="22"/>
+      <c r="AB4" s="22"/>
+      <c r="AC4" s="22"/>
+      <c r="AD4" s="22"/>
+      <c r="AE4" s="22"/>
+      <c r="AF4" s="23">
         <f t="shared" ref="AF4" si="0">+SUM($M4:$AE4)</f>
         <v>0</v>
       </c>
-      <c r="AG4" s="29"/>
-      <c r="AH4" s="27"/>
-      <c r="AI4" s="27"/>
-      <c r="AJ4" s="27"/>
-      <c r="AK4" s="27"/>
-      <c r="AL4" s="27"/>
-      <c r="AM4" s="27"/>
-      <c r="AN4" s="28">
+      <c r="AG4" s="24"/>
+      <c r="AH4" s="22"/>
+      <c r="AI4" s="22"/>
+      <c r="AJ4" s="22"/>
+      <c r="AK4" s="22"/>
+      <c r="AL4" s="22"/>
+      <c r="AM4" s="22"/>
+      <c r="AN4" s="23">
         <f t="shared" ref="AN4" si="1">SUM($AH4:$AM4)</f>
         <v>0</v>
       </c>
-      <c r="AP4" s="27"/>
-      <c r="AQ4" s="27"/>
-      <c r="AR4" s="27"/>
-      <c r="AS4" s="28">
+      <c r="AP4" s="22"/>
+      <c r="AQ4" s="22"/>
+      <c r="AR4" s="22"/>
+      <c r="AS4" s="23">
         <f t="shared" ref="AS4" si="2">SUM($AP4:$AR4)</f>
         <v>0</v>
       </c>
-      <c r="AT4" s="30">
+      <c r="AT4" s="25">
         <f t="shared" ref="AT4" si="3">SUM(AN4,AS4)</f>
         <v>0</v>
       </c>
-      <c r="AU4" s="27"/>
-      <c r="AV4" s="27"/>
-      <c r="AW4" s="27"/>
-      <c r="AX4" s="27"/>
-      <c r="AY4" s="27"/>
-      <c r="AZ4" s="31">
+      <c r="AU4" s="22"/>
+      <c r="AV4" s="22"/>
+      <c r="AW4" s="22"/>
+      <c r="AX4" s="22"/>
+      <c r="AY4" s="22"/>
+      <c r="AZ4" s="26">
         <f t="shared" ref="AZ4" si="4">SUM($AU4:$AY4)</f>
         <v>0</v>
       </c>
-      <c r="BA4" s="29"/>
-      <c r="BB4" s="27">
+      <c r="BA4" s="24"/>
+      <c r="BB4" s="22">
         <f t="shared" ref="BB4" si="5">SUM($AF4,$AN4,$AS4,$AZ4)+BD4</f>
         <v>0</v>
       </c>
-      <c r="BC4" s="27">
+      <c r="BC4" s="22">
         <f t="shared" ref="BC4" si="6">120*$BG4</f>
         <v>0</v>
       </c>
-      <c r="BD4" s="27">
+      <c r="BD4" s="22">
         <f t="shared" ref="BD4" si="7">SUM($AF4,$AN4,$AS4,$AZ4)*0.4%</f>
         <v>0</v>
       </c>
-      <c r="BE4" s="27">
+      <c r="BE4" s="22">
         <f t="shared" ref="BE4" si="8">$BC4*19%</f>
         <v>0</v>
       </c>
-      <c r="BF4" s="27">
+      <c r="BF4" s="22">
         <f>SUM(BB4,BC4,BE4)</f>
         <v>0</v>
       </c>
-      <c r="BG4" s="32"/>
-      <c r="BH4" s="33" t="e">
+      <c r="BG4" s="27"/>
+      <c r="BH4" s="28" t="e">
         <f t="shared" ref="BH4" si="9">ROUND($BB4/$BG4,2)</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="BI4" s="33" t="e">
+      <c r="BI4" s="28" t="e">
         <f t="shared" ref="BI4" si="10">ROUND($BC4/$BG4,2)</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="BJ4" s="33" t="e">
+      <c r="BJ4" s="28" t="e">
         <f t="shared" ref="BJ4" si="11">ROUND($BE4/$BG4,2)</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="BK4" s="33" t="e">
+      <c r="BK4" s="28" t="e">
         <f t="shared" ref="BK4" si="12">SUM($BH4:$BJ4)</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="BL4" s="34"/>
-      <c r="BM4" s="33" t="e">
+      <c r="BL4" s="29"/>
+      <c r="BM4" s="28" t="e">
         <f t="shared" ref="BM4" si="13">BK4-BL4</f>
         <v>#DIV/0!</v>
       </c>
     </row>
     <row r="5" spans="1:65" x14ac:dyDescent="0.3">
-      <c r="A5" s="35"/>
-      <c r="B5" s="35"/>
-      <c r="C5" s="35" t="s">
+      <c r="A5" s="30"/>
+      <c r="B5" s="30"/>
+      <c r="C5" s="30" t="s">
         <v>65</v>
       </c>
-      <c r="D5" s="35"/>
-      <c r="E5" s="35"/>
-      <c r="F5" s="35"/>
-      <c r="G5" s="35"/>
-      <c r="H5" s="36" t="s">
+      <c r="D5" s="30"/>
+      <c r="E5" s="30"/>
+      <c r="F5" s="30"/>
+      <c r="G5" s="30"/>
+      <c r="H5" s="31" t="s">
         <v>65</v>
       </c>
-      <c r="I5" s="36"/>
-      <c r="J5" s="36"/>
-      <c r="K5" s="36"/>
-      <c r="L5" s="36"/>
-      <c r="M5" s="37">
+      <c r="I5" s="31"/>
+      <c r="J5" s="31"/>
+      <c r="K5" s="31"/>
+      <c r="L5" s="31"/>
+      <c r="M5" s="32">
         <f t="shared" ref="M5:AF5" si="14">SUM(M4:M4)</f>
         <v>0</v>
       </c>
-      <c r="N5" s="37">
-        <f t="shared" si="14"/>
-        <v>0</v>
-      </c>
-      <c r="O5" s="37">
-        <f t="shared" si="14"/>
-        <v>0</v>
-      </c>
-      <c r="P5" s="37">
-        <f t="shared" si="14"/>
-        <v>0</v>
-      </c>
-      <c r="Q5" s="37">
-        <f t="shared" si="14"/>
-        <v>0</v>
-      </c>
-      <c r="R5" s="37">
-        <f t="shared" si="14"/>
-        <v>0</v>
-      </c>
-      <c r="S5" s="37">
-        <f t="shared" si="14"/>
-        <v>0</v>
-      </c>
-      <c r="T5" s="37">
-        <f t="shared" si="14"/>
-        <v>0</v>
-      </c>
-      <c r="U5" s="37">
-        <f t="shared" si="14"/>
-        <v>0</v>
-      </c>
-      <c r="V5" s="37">
-        <f t="shared" si="14"/>
-        <v>0</v>
-      </c>
-      <c r="W5" s="37">
-        <f t="shared" si="14"/>
-        <v>0</v>
-      </c>
-      <c r="X5" s="37">
-        <f t="shared" si="14"/>
-        <v>0</v>
-      </c>
-      <c r="Y5" s="37">
-        <f t="shared" si="14"/>
-        <v>0</v>
-      </c>
-      <c r="Z5" s="37">
-        <f t="shared" si="14"/>
-        <v>0</v>
-      </c>
-      <c r="AA5" s="37">
-        <f t="shared" si="14"/>
-        <v>0</v>
-      </c>
-      <c r="AB5" s="37">
-        <f t="shared" si="14"/>
-        <v>0</v>
-      </c>
-      <c r="AC5" s="37">
-        <f t="shared" si="14"/>
-        <v>0</v>
-      </c>
-      <c r="AD5" s="37">
-        <f t="shared" si="14"/>
-        <v>0</v>
-      </c>
-      <c r="AE5" s="37">
-        <f t="shared" si="14"/>
-        <v>0</v>
-      </c>
-      <c r="AF5" s="37">
-        <f t="shared" si="14"/>
-        <v>0</v>
-      </c>
-      <c r="AG5" s="29"/>
-      <c r="AH5" s="37">
+      <c r="N5" s="32">
+        <f t="shared" si="14"/>
+        <v>0</v>
+      </c>
+      <c r="O5" s="32">
+        <f t="shared" si="14"/>
+        <v>0</v>
+      </c>
+      <c r="P5" s="32">
+        <f t="shared" si="14"/>
+        <v>0</v>
+      </c>
+      <c r="Q5" s="32">
+        <f t="shared" si="14"/>
+        <v>0</v>
+      </c>
+      <c r="R5" s="32">
+        <f t="shared" si="14"/>
+        <v>0</v>
+      </c>
+      <c r="S5" s="32">
+        <f t="shared" si="14"/>
+        <v>0</v>
+      </c>
+      <c r="T5" s="32">
+        <f t="shared" si="14"/>
+        <v>0</v>
+      </c>
+      <c r="U5" s="32">
+        <f t="shared" si="14"/>
+        <v>0</v>
+      </c>
+      <c r="V5" s="32">
+        <f t="shared" si="14"/>
+        <v>0</v>
+      </c>
+      <c r="W5" s="32">
+        <f t="shared" si="14"/>
+        <v>0</v>
+      </c>
+      <c r="X5" s="32">
+        <f t="shared" si="14"/>
+        <v>0</v>
+      </c>
+      <c r="Y5" s="32">
+        <f t="shared" si="14"/>
+        <v>0</v>
+      </c>
+      <c r="Z5" s="32">
+        <f t="shared" si="14"/>
+        <v>0</v>
+      </c>
+      <c r="AA5" s="32">
+        <f t="shared" si="14"/>
+        <v>0</v>
+      </c>
+      <c r="AB5" s="32">
+        <f t="shared" si="14"/>
+        <v>0</v>
+      </c>
+      <c r="AC5" s="32">
+        <f t="shared" si="14"/>
+        <v>0</v>
+      </c>
+      <c r="AD5" s="32">
+        <f t="shared" si="14"/>
+        <v>0</v>
+      </c>
+      <c r="AE5" s="32">
+        <f t="shared" si="14"/>
+        <v>0</v>
+      </c>
+      <c r="AF5" s="32">
+        <f t="shared" si="14"/>
+        <v>0</v>
+      </c>
+      <c r="AG5" s="24"/>
+      <c r="AH5" s="32">
         <f t="shared" ref="AH5:AN5" si="15">SUM(AH4:AH4)</f>
         <v>0</v>
       </c>
-      <c r="AI5" s="37">
+      <c r="AI5" s="32">
         <f t="shared" si="15"/>
         <v>0</v>
       </c>
-      <c r="AJ5" s="37">
+      <c r="AJ5" s="32">
         <f t="shared" si="15"/>
         <v>0</v>
       </c>
-      <c r="AK5" s="37">
+      <c r="AK5" s="32">
         <f t="shared" si="15"/>
         <v>0</v>
       </c>
-      <c r="AL5" s="37">
+      <c r="AL5" s="32">
         <f t="shared" si="15"/>
         <v>0</v>
       </c>
-      <c r="AM5" s="37">
+      <c r="AM5" s="32">
         <f t="shared" si="15"/>
         <v>0</v>
       </c>
-      <c r="AN5" s="37">
+      <c r="AN5" s="32">
         <f t="shared" si="15"/>
         <v>0</v>
       </c>
-      <c r="AP5" s="37">
+      <c r="AP5" s="32">
         <f>SUM(AP4:AP4)</f>
         <v>0</v>
       </c>
-      <c r="AQ5" s="37">
+      <c r="AQ5" s="32">
         <f>SUM(AQ4:AQ4)</f>
         <v>0</v>
       </c>
-      <c r="AR5" s="37">
+      <c r="AR5" s="32">
         <f>SUM(AR4:AR4)</f>
         <v>0</v>
       </c>
-      <c r="AS5" s="37">
+      <c r="AS5" s="32">
         <f>SUM(AS4:AS4)</f>
         <v>0</v>
       </c>
-      <c r="AT5" s="38"/>
-      <c r="AU5" s="37">
+      <c r="AT5" s="33"/>
+      <c r="AU5" s="32">
         <f t="shared" ref="AU5:AZ5" si="16">SUM(AU4:AU4)</f>
         <v>0</v>
       </c>
-      <c r="AV5" s="37">
+      <c r="AV5" s="32">
         <f t="shared" si="16"/>
         <v>0</v>
       </c>
-      <c r="AW5" s="37">
+      <c r="AW5" s="32">
         <f t="shared" si="16"/>
         <v>0</v>
       </c>
-      <c r="AX5" s="37">
+      <c r="AX5" s="32">
         <f t="shared" si="16"/>
         <v>0</v>
       </c>
-      <c r="AY5" s="37">
+      <c r="AY5" s="32">
         <f t="shared" si="16"/>
         <v>0</v>
       </c>
-      <c r="AZ5" s="37">
+      <c r="AZ5" s="32">
         <f t="shared" si="16"/>
         <v>0</v>
       </c>
-      <c r="BA5" s="29"/>
-      <c r="BB5" s="37">
+      <c r="BA5" s="24"/>
+      <c r="BB5" s="32">
         <f>SUM(BB4:BB4)</f>
         <v>0</v>
       </c>
-      <c r="BC5" s="37">
+      <c r="BC5" s="32">
         <f>SUM(BC4:BC4)</f>
         <v>0</v>
       </c>
-      <c r="BD5" s="37">
+      <c r="BD5" s="32">
         <f>SUM(BD4:BD4)</f>
         <v>0</v>
       </c>
-      <c r="BE5" s="37">
+      <c r="BE5" s="32">
         <f>SUM(BE4:BE4)</f>
         <v>0</v>
       </c>
-      <c r="BF5" s="37">
+      <c r="BF5" s="32">
         <f>SUM(BF4:BF4)</f>
         <v>0</v>
       </c>
-      <c r="BG5" s="37"/>
-      <c r="BH5" s="39" t="e">
+      <c r="BG5" s="32"/>
+      <c r="BH5" s="34" t="e">
         <f>SUM(BH4:BH4)</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="BI5" s="39" t="e">
+      <c r="BI5" s="34" t="e">
         <f>SUM(BI4:BI4)</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="BJ5" s="39" t="e">
+      <c r="BJ5" s="34" t="e">
         <f>SUM(BJ4:BJ4)</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="BK5" s="39" t="e">
+      <c r="BK5" s="34" t="e">
         <f>SUM(BK4:BK4)</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="BL5" s="34"/>
-      <c r="BM5" s="33" t="e">
+      <c r="BL5" s="29"/>
+      <c r="BM5" s="28" t="e">
         <f>BK5-BL5</f>
         <v>#DIV/0!</v>
       </c>
     </row>
     <row r="7" spans="1:65" x14ac:dyDescent="0.3">
-      <c r="A7" s="40" t="s">
+      <c r="A7" s="35" t="s">
         <v>66</v>
       </c>
-      <c r="R7" s="41"/>
+      <c r="R7" s="36"/>
     </row>
   </sheetData>
   <mergeCells count="4">

</xml_diff>